<commit_message>
Drop PL nr. from UK/Battery cost summary detail sheet
The matching in this report is by customer name only (these Backlog
lines have no shipment number yet) — showing Q3's internal "PL nr."
reference in the detail sheet was mistaken for shipment-number matching.
Removed it; the join key was never SH#/PL nr.
</commit_message>
<xml_diff>
--- a/output/UK_Battery_Cost_Summary.xlsx
+++ b/output/UK_Battery_Cost_Summary.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$1:$F$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Q3 Detail'!$A$1:$G$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Q3 Detail'!$A$1:$F$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1032,16 +1032,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1057,25 +1056,20 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>PL nr.</t>
+          <t>Country</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Country</t>
+          <t>Nr. of pal</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Nr. of pal</t>
+          <t>Solaredge rate (EUR)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Solaredge rate (EUR)</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Solaredge rate (USD)</t>
         </is>
@@ -1094,21 +1088,16 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>SH215202619644</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
           <t>Italy</t>
         </is>
       </c>
+      <c r="D2" s="2" t="n">
+        <v>12</v>
+      </c>
       <c r="E2" s="2" t="n">
-        <v>12</v>
+        <v>3990</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>3990</v>
-      </c>
-      <c r="G2" s="2" t="n">
         <v>4635.58</v>
       </c>
     </row>
@@ -1125,21 +1114,16 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>SH215202619237</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D3" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="E3" s="2" t="n">
-        <v>9</v>
+        <v>3890</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>3890</v>
-      </c>
-      <c r="G3" s="2" t="n">
         <v>4519.4</v>
       </c>
     </row>
@@ -1156,21 +1140,16 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>SH215202619238</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D4" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="E4" s="2" t="n">
-        <v>2</v>
+        <v>1750</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1750</v>
-      </c>
-      <c r="G4" s="2" t="n">
         <v>2033.15</v>
       </c>
     </row>
@@ -1187,21 +1166,16 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>SH108202619159</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D5" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="E5" s="2" t="n">
-        <v>2</v>
+        <v>2600</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>2600</v>
-      </c>
-      <c r="G5" s="2" t="n">
         <v>3020.68</v>
       </c>
     </row>
@@ -1218,19 +1192,14 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>SH108202619184</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="D6" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1245,21 +1214,16 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>SH215202619450</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D7" s="2" t="n">
+        <v>11</v>
+      </c>
       <c r="E7" s="2" t="n">
-        <v>11</v>
+        <v>2600</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>2600</v>
-      </c>
-      <c r="G7" s="2" t="n">
         <v>3020.68</v>
       </c>
     </row>
@@ -1276,21 +1240,16 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>SH108202619517</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D8" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="E8" s="2" t="n">
-        <v>1</v>
+        <v>1550</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>1550</v>
-      </c>
-      <c r="G8" s="2" t="n">
         <v>1800.79</v>
       </c>
     </row>
@@ -1307,21 +1266,16 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>SH108202619474</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D9" s="2" t="n">
+        <v>30</v>
+      </c>
       <c r="E9" s="2" t="n">
-        <v>30</v>
+        <v>3690</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>3690</v>
-      </c>
-      <c r="G9" s="2" t="n">
         <v>4287.04</v>
       </c>
     </row>
@@ -1338,21 +1292,16 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>SH108202619599</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D10" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="E10" s="2" t="n">
-        <v>8</v>
+        <v>2350</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>2350</v>
-      </c>
-      <c r="G10" s="2" t="n">
         <v>2730.23</v>
       </c>
     </row>
@@ -1369,21 +1318,16 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>SH215202619648</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D11" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="E11" s="2" t="n">
-        <v>1</v>
+        <v>1590</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>1590</v>
-      </c>
-      <c r="G11" s="2" t="n">
         <v>1847.26</v>
       </c>
     </row>
@@ -1400,21 +1344,16 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>SH108202619637</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D12" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="E12" s="2" t="n">
-        <v>1</v>
+        <v>1590</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>1590</v>
-      </c>
-      <c r="G12" s="2" t="n">
         <v>1847.26</v>
       </c>
     </row>
@@ -1431,21 +1370,16 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>SH215202619236</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
           <t>Italy</t>
         </is>
       </c>
+      <c r="D13" s="2" t="n">
+        <v>20</v>
+      </c>
       <c r="E13" s="2" t="n">
-        <v>20</v>
+        <v>3690</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>3690</v>
-      </c>
-      <c r="G13" s="2" t="n">
         <v>4287.04</v>
       </c>
     </row>
@@ -1462,21 +1396,16 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>SH215202619464</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
           <t>France</t>
         </is>
       </c>
+      <c r="D14" s="2" t="n">
+        <v>19</v>
+      </c>
       <c r="E14" s="2" t="n">
-        <v>19</v>
+        <v>3750</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>3750</v>
-      </c>
-      <c r="G14" s="2" t="n">
         <v>4356.75</v>
       </c>
     </row>
@@ -1493,21 +1422,16 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>SH108202619307</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D15" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E15" s="2" t="n">
-        <v>3</v>
+        <v>1950</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>1950</v>
-      </c>
-      <c r="G15" s="2" t="n">
         <v>2265.51</v>
       </c>
     </row>
@@ -1524,21 +1448,16 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>SH215202619253</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D16" s="2" t="n">
+        <v>25</v>
+      </c>
       <c r="E16" s="2" t="n">
-        <v>25</v>
+        <v>4050</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>4050</v>
-      </c>
-      <c r="G16" s="2" t="n">
         <v>4705.29</v>
       </c>
     </row>
@@ -1555,21 +1474,16 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>SH215202619268</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D17" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="E17" s="2" t="n">
-        <v>9</v>
+        <v>2690</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>2690</v>
-      </c>
-      <c r="G17" s="2" t="n">
         <v>3125.24</v>
       </c>
     </row>
@@ -1586,21 +1500,16 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>SH108202619325</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D18" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="E18" s="2" t="n">
-        <v>5</v>
+        <v>1920</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>1920</v>
-      </c>
-      <c r="G18" s="2" t="n">
         <v>2230.66</v>
       </c>
     </row>
@@ -1617,21 +1526,16 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>SH108202619396</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D19" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="E19" s="2" t="n">
-        <v>5</v>
+        <v>1920</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>1920</v>
-      </c>
-      <c r="G19" s="2" t="n">
         <v>2230.66</v>
       </c>
     </row>
@@ -1648,21 +1552,16 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>SH215202619459</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D20" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="E20" s="2" t="n">
-        <v>1</v>
+        <v>1550</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>1550</v>
-      </c>
-      <c r="G20" s="2" t="n">
         <v>1800.79</v>
       </c>
     </row>
@@ -1679,21 +1578,16 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>SH108202619492</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D21" s="2" t="n">
+        <v>11</v>
+      </c>
       <c r="E21" s="2" t="n">
-        <v>11</v>
+        <v>2950</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>2950</v>
-      </c>
-      <c r="G21" s="2" t="n">
         <v>3427.31</v>
       </c>
     </row>
@@ -1710,21 +1604,16 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>SH108202619493</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D22" s="2" t="n">
+        <v>23</v>
+      </c>
       <c r="E22" s="2" t="n">
-        <v>23</v>
+        <v>3800</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>3800</v>
-      </c>
-      <c r="G22" s="2" t="n">
         <v>4414.84</v>
       </c>
     </row>
@@ -1741,21 +1630,16 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>SH215202619573</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D23" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="E23" s="2" t="n">
-        <v>8</v>
+        <v>2830</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>2830</v>
-      </c>
-      <c r="G23" s="2" t="n">
         <v>3287.89</v>
       </c>
     </row>
@@ -1772,21 +1656,16 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>SH215202619433</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D24" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="E24" s="2" t="n">
-        <v>1</v>
+        <v>1550</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>1550</v>
-      </c>
-      <c r="G24" s="2" t="n">
         <v>1800.79</v>
       </c>
     </row>
@@ -1803,21 +1682,16 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>SH108202619615</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D25" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="E25" s="2" t="n">
-        <v>2</v>
+        <v>1590</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>1590</v>
-      </c>
-      <c r="G25" s="2" t="n">
         <v>1847.26</v>
       </c>
     </row>
@@ -1834,21 +1708,16 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>SH108202619631</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D26" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="E26" s="2" t="n">
-        <v>1</v>
+        <v>1550</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>1550</v>
-      </c>
-      <c r="G26" s="2" t="n">
         <v>1800.79</v>
       </c>
     </row>
@@ -1865,21 +1734,16 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>SH215202619722</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D27" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="E27" s="2" t="n">
-        <v>1</v>
+        <v>1590</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>1590</v>
-      </c>
-      <c r="G27" s="2" t="n">
         <v>1847.26</v>
       </c>
     </row>
@@ -1896,21 +1760,16 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>SH215202619374</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
           <t>Germany</t>
         </is>
       </c>
+      <c r="D28" s="2" t="n">
+        <v>17</v>
+      </c>
       <c r="E28" s="2" t="n">
-        <v>17</v>
+        <v>2990</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>2990</v>
-      </c>
-      <c r="G28" s="2" t="n">
         <v>3473.78</v>
       </c>
     </row>
@@ -1927,21 +1786,16 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>SH215202619536</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
           <t>Germany</t>
         </is>
       </c>
+      <c r="D29" s="2" t="n">
+        <v>11</v>
+      </c>
       <c r="E29" s="2" t="n">
-        <v>11</v>
+        <v>2990</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>2990</v>
-      </c>
-      <c r="G29" s="2" t="n">
         <v>3473.78</v>
       </c>
     </row>
@@ -1958,21 +1812,16 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>SH215202619257</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
           <t>Poland</t>
         </is>
       </c>
+      <c r="D30" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="E30" s="2" t="n">
-        <v>2</v>
+        <v>2200</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>2200</v>
-      </c>
-      <c r="G30" s="2" t="n">
         <v>2555.96</v>
       </c>
     </row>
@@ -1989,21 +1838,16 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>SH215202619449</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
           <t>Poland</t>
         </is>
       </c>
+      <c r="D31" s="2" t="n">
+        <v>7</v>
+      </c>
       <c r="E31" s="2" t="n">
-        <v>7</v>
+        <v>2600</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>2600</v>
-      </c>
-      <c r="G31" s="2" t="n">
         <v>3020.68</v>
       </c>
     </row>
@@ -2020,21 +1864,16 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>SH215202619533</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
           <t>Poland</t>
         </is>
       </c>
+      <c r="D32" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E32" s="2" t="n">
-        <v>3</v>
+        <v>2350</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>2350</v>
-      </c>
-      <c r="G32" s="2" t="n">
         <v>2730.23</v>
       </c>
     </row>
@@ -2051,21 +1890,16 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>SH215202619369</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
           <t>Switzerland</t>
         </is>
       </c>
+      <c r="D33" s="2" t="n">
+        <v>33</v>
+      </c>
       <c r="E33" s="2" t="n">
-        <v>33</v>
+        <v>3500</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>3500</v>
-      </c>
-      <c r="G33" s="2" t="n">
         <v>4066.3</v>
       </c>
     </row>
@@ -2082,21 +1916,16 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>SH215202619531</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
           <t>Switzerland</t>
         </is>
       </c>
+      <c r="D34" s="2" t="n">
+        <v>33</v>
+      </c>
       <c r="E34" s="2" t="n">
-        <v>33</v>
+        <v>4050</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>4050</v>
-      </c>
-      <c r="G34" s="2" t="n">
         <v>4705.29</v>
       </c>
     </row>
@@ -2113,21 +1942,16 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>SH215202619538</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
           <t>Switzerland</t>
         </is>
       </c>
+      <c r="D35" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="E35" s="2" t="n">
-        <v>9</v>
+        <v>2590</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>2590</v>
-      </c>
-      <c r="G35" s="2" t="n">
         <v>3009.06</v>
       </c>
     </row>
@@ -2144,21 +1968,16 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>SH215202619530</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
           <t>Germany</t>
         </is>
       </c>
+      <c r="D36" s="2" t="n">
+        <v>33</v>
+      </c>
       <c r="E36" s="2" t="n">
-        <v>33</v>
+        <v>3050</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>3050</v>
-      </c>
-      <c r="G36" s="2" t="n">
         <v>3543.49</v>
       </c>
     </row>
@@ -2175,21 +1994,16 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>SH215202619537</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
           <t>Germany</t>
         </is>
       </c>
+      <c r="D37" s="2" t="n">
+        <v>33</v>
+      </c>
       <c r="E37" s="2" t="n">
-        <v>33</v>
+        <v>3050</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>3050</v>
-      </c>
-      <c r="G37" s="2" t="n">
         <v>3543.49</v>
       </c>
     </row>
@@ -2206,21 +2020,16 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>SH215202619321</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
           <t>Germany</t>
         </is>
       </c>
+      <c r="D38" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="E38" s="2" t="n">
-        <v>13</v>
+        <v>2390</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>2390</v>
-      </c>
-      <c r="G38" s="2" t="n">
         <v>2776.7</v>
       </c>
     </row>
@@ -2237,21 +2046,16 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>SH215202619263</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
           <t>Germany</t>
         </is>
       </c>
+      <c r="D39" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="E39" s="2" t="n">
-        <v>13</v>
+        <v>3050</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>3050</v>
-      </c>
-      <c r="G39" s="2" t="n">
         <v>3543.49</v>
       </c>
     </row>
@@ -2268,21 +2072,16 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>SH215202619373</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
           <t>Germany</t>
         </is>
       </c>
+      <c r="D40" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="E40" s="2" t="n">
-        <v>13</v>
+        <v>2400</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>2400</v>
-      </c>
-      <c r="G40" s="2" t="n">
         <v>2788.32</v>
       </c>
     </row>
@@ -2299,21 +2098,16 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>SH215202619655</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
           <t>Germany</t>
         </is>
       </c>
+      <c r="D41" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="E41" s="2" t="n">
-        <v>13</v>
+        <v>2390</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>2390</v>
-      </c>
-      <c r="G41" s="2" t="n">
         <v>2776.7</v>
       </c>
     </row>
@@ -2330,21 +2124,16 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>SH215202619455</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
           <t>Netherlands</t>
         </is>
       </c>
+      <c r="D42" s="2" t="n">
+        <v>22</v>
+      </c>
       <c r="E42" s="2" t="n">
-        <v>22</v>
+        <v>1990</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>1990</v>
-      </c>
-      <c r="G42" s="2" t="n">
         <v>2311.98</v>
       </c>
     </row>
@@ -2361,21 +2150,16 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>SH215202619518</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
           <t>Austria</t>
         </is>
       </c>
+      <c r="D43" s="2" t="n">
+        <v>25</v>
+      </c>
       <c r="E43" s="2" t="n">
-        <v>25</v>
+        <v>3990</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>3990</v>
-      </c>
-      <c r="G43" s="2" t="n">
         <v>4635.58</v>
       </c>
     </row>
@@ -2392,21 +2176,16 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>SH215202619532</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
           <t>Austria</t>
         </is>
       </c>
+      <c r="D44" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="E44" s="2" t="n">
-        <v>13</v>
+        <v>2990</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>2990</v>
-      </c>
-      <c r="G44" s="2" t="n">
         <v>3473.78</v>
       </c>
     </row>
@@ -2423,21 +2202,16 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>SH215202619581</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
           <t>Austria</t>
         </is>
       </c>
+      <c r="D45" s="2" t="n">
+        <v>33</v>
+      </c>
       <c r="E45" s="2" t="n">
-        <v>33</v>
+        <v>3990</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>3990</v>
-      </c>
-      <c r="G45" s="2" t="n">
         <v>4635.58</v>
       </c>
     </row>
@@ -2454,21 +2228,16 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>SH215202619584</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
           <t>Austria</t>
         </is>
       </c>
+      <c r="D46" s="2" t="n">
+        <v>11</v>
+      </c>
       <c r="E46" s="2" t="n">
-        <v>11</v>
+        <v>3990</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>3990</v>
-      </c>
-      <c r="G46" s="2" t="n">
         <v>4635.58</v>
       </c>
     </row>
@@ -2485,21 +2254,16 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>SH215202619240</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
           <t>Netherlands</t>
         </is>
       </c>
+      <c r="D47" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="E47" s="2" t="n">
-        <v>4</v>
+        <v>2050</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>2050</v>
-      </c>
-      <c r="G47" s="2" t="n">
         <v>2381.69</v>
       </c>
     </row>
@@ -2516,19 +2280,14 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>SH215202619322</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
           <t>Netherlands</t>
         </is>
       </c>
-      <c r="E48" s="2" t="n">
+      <c r="D48" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="n"/>
-      <c r="G48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2543,21 +2302,16 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>SH215202619568</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
           <t>Netherlands</t>
         </is>
       </c>
+      <c r="D49" s="2" t="n">
+        <v>12</v>
+      </c>
       <c r="E49" s="2" t="n">
-        <v>12</v>
+        <v>1990</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>1990</v>
-      </c>
-      <c r="G49" s="2" t="n">
         <v>2311.98</v>
       </c>
     </row>
@@ -2574,21 +2328,16 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>SH215202619591</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
           <t>Netherlands</t>
         </is>
       </c>
+      <c r="D50" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="E50" s="2" t="n">
-        <v>6</v>
+        <v>1990</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>1990</v>
-      </c>
-      <c r="G50" s="2" t="n">
         <v>2311.98</v>
       </c>
     </row>
@@ -2605,21 +2354,16 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>SH215202619717</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
           <t>Netherlands</t>
         </is>
       </c>
+      <c r="D51" s="2" t="n">
+        <v>12</v>
+      </c>
       <c r="E51" s="2" t="n">
-        <v>12</v>
+        <v>1990</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>1990</v>
-      </c>
-      <c r="G51" s="2" t="n">
         <v>2311.98</v>
       </c>
     </row>
@@ -2636,21 +2380,16 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>SH215202619465</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
           <t>Italy</t>
         </is>
       </c>
+      <c r="D52" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="E52" s="2" t="n">
-        <v>2</v>
+        <v>4300</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>4300</v>
-      </c>
-      <c r="G52" s="2" t="n">
         <v>4995.74</v>
       </c>
     </row>
@@ -2667,21 +2406,16 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>SH108202619480</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D53" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="E53" s="2" t="n">
-        <v>1</v>
+        <v>1550</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>1550</v>
-      </c>
-      <c r="G53" s="2" t="n">
         <v>1800.79</v>
       </c>
     </row>
@@ -2698,21 +2432,16 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>SH215202619454</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D54" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="E54" s="2" t="n">
-        <v>1</v>
+        <v>1550</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>1550</v>
-      </c>
-      <c r="G54" s="2" t="n">
         <v>1800.79</v>
       </c>
     </row>
@@ -2729,21 +2458,16 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>SH108202619606</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D55" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E55" s="2" t="n">
-        <v>3</v>
+        <v>1790</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>1790</v>
-      </c>
-      <c r="G55" s="2" t="n">
         <v>2079.62</v>
       </c>
     </row>
@@ -2760,21 +2484,16 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>SH215202619246</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
           <t>Switzerland</t>
         </is>
       </c>
+      <c r="D56" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="E56" s="2" t="n">
-        <v>10</v>
+        <v>2600</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>2600</v>
-      </c>
-      <c r="G56" s="2" t="n">
         <v>3020.68</v>
       </c>
     </row>
@@ -2791,21 +2510,16 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>SH215202619247</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
           <t>Switzerland</t>
         </is>
       </c>
+      <c r="D57" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="E57" s="2" t="n">
-        <v>4</v>
+        <v>2090</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>2090</v>
-      </c>
-      <c r="G57" s="2" t="n">
         <v>2428.16</v>
       </c>
     </row>
@@ -2822,21 +2536,16 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>SH215202619366</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
           <t>Switzerland</t>
         </is>
       </c>
+      <c r="D58" s="2" t="n">
+        <v>14</v>
+      </c>
       <c r="E58" s="2" t="n">
-        <v>14</v>
+        <v>3300</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>3300</v>
-      </c>
-      <c r="G58" s="2" t="n">
         <v>3833.94</v>
       </c>
     </row>
@@ -2853,21 +2562,16 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>SH215202619529</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
           <t>Switzerland</t>
         </is>
       </c>
+      <c r="D59" s="2" t="n">
+        <v>26</v>
+      </c>
       <c r="E59" s="2" t="n">
-        <v>26</v>
+        <v>3550</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>3550</v>
-      </c>
-      <c r="G59" s="2" t="n">
         <v>4124.39</v>
       </c>
     </row>
@@ -2884,21 +2588,16 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>SH108202619556</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="D60" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="E60" s="2" t="n">
-        <v>8</v>
+        <v>2190</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>2190</v>
-      </c>
-      <c r="G60" s="2" t="n">
         <v>2544.34</v>
       </c>
     </row>
@@ -2915,21 +2614,16 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>SH215202619440</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
           <t>Switzerland</t>
         </is>
       </c>
+      <c r="D61" s="2" t="n">
+        <v>17</v>
+      </c>
       <c r="E61" s="2" t="n">
-        <v>17</v>
+        <v>3400</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>3400</v>
-      </c>
-      <c r="G61" s="2" t="n">
         <v>3950.12</v>
       </c>
     </row>
@@ -2946,21 +2640,16 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> SH215202619583</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
           <t>Switzerland</t>
         </is>
       </c>
+      <c r="D62" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="E62" s="2" t="n">
-        <v>1</v>
+        <v>2050</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>2050</v>
-      </c>
-      <c r="G62" s="2" t="n">
         <v>2381.69</v>
       </c>
     </row>
@@ -2977,21 +2666,16 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>SH215202619239</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
           <t>Germany</t>
         </is>
       </c>
+      <c r="D63" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="E63" s="2" t="n">
-        <v>10</v>
+        <v>2400</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>2400</v>
-      </c>
-      <c r="G63" s="2" t="n">
         <v>2788.32</v>
       </c>
     </row>
@@ -3008,26 +2692,21 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>SH215202619526</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
           <t>Germany</t>
         </is>
       </c>
+      <c r="D64" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="E64" s="2" t="n">
-        <v>2</v>
+        <v>1990</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>1990</v>
-      </c>
-      <c r="G64" s="2" t="n">
         <v>2311.98</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G64"/>
+  <autoFilter ref="A1:F64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>